<commit_message>
Day 2 lab: add combination experiment T21 (val only), update report, results.xlsx and README
T21 = class-weighted CE + CutMix + EMA, 3 seeds: val macro-F1 0.9600 +/- 0.0010 vs T00 0.9710 +/- 0.0042
(effects do not add up). No test data touched; final F01 unchanged.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/submissions/2A202602985_ngo_duc_chung/results.xlsx
+++ b/submissions/2A202602985_ngo_duc_chung/results.xlsx
@@ -1078,15 +1078,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
@@ -2162,6 +2162,226 @@
       <c r="N19" t="inlineStr">
         <is>
           <t>F01 seed 0 chính là T00 seed 0 + EMA (EMA không đổi quá trình huấn luyện, chỉ đổi trọng số đánh giá); tương ứng ablation T16 của lượt 1; không phân biệt được với nhiễu (σ T00 cùng lượt = 0.0042)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>T21</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Kaggle T4 (lượt 3, chỉ T21)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>kết hợp (C+B+F)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>CE trọng số lớp + CutMix + EMA 0.99</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>0.9610382149685707</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>0.9682947729220223</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>-0.005255182253908752</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>-1.253992650681643</v>
+      </c>
+      <c r="K20" s="2" t="n">
+        <v>-0.009969375377865242</v>
+      </c>
+      <c r="L20" s="2" t="n">
+        <v>0.9513274336283186</v>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>0.9039812646370023</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>tổ hợp; Δ so với T00 cùng seed = -0.0053</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>T21</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Kaggle T4 (lượt 3, chỉ T21)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>kết hợp (C+B+F)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>CE trọng số lớp + CutMix + EMA 0.99</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>0.9600961762475035</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>0.9680091402456441</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>-0.006197220974975881</v>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>-1.478782120542002</v>
+      </c>
+      <c r="K21" s="2" t="n">
+        <v>-0.01091141409893237</v>
+      </c>
+      <c r="L21" s="2" t="n">
+        <v>0.9303370786516855</v>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>0.8981481481481481</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>tổ hợp; Δ so với T00 cùng seed = -0.0123</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>T21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Kaggle T4 (lượt 3, chỉ T21)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>kết hợp (C+B+F)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>CE trọng số lớp + CutMix + EMA 0.99</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>0.9590056247620967</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>0.9657240788346186</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>-0.007287772460382702</v>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>-1.7390097362204</v>
+      </c>
+      <c r="K22" s="2" t="n">
+        <v>-0.01200196558433919</v>
+      </c>
+      <c r="L22" s="2" t="n">
+        <v>0.9406593406593408</v>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>0.909952606635071</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>tổ hợp; Δ so với T00 cùng seed = -0.0153</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>T21 (mean ± std, 3 seed)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Kaggle T4 (lượt 3, chỉ T21)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>kết hợp (C+B+F)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>CE trọng số lớp + CutMix + EMA 0.99</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>0,1,2</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>0.9600466719927235</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>0.9673426640007617</v>
+      </c>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="n">
+        <v>-2.615496551057489</v>
+      </c>
+      <c r="K23" s="2" t="n">
+        <v>-0.01096091835371238</v>
+      </c>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>mean macro-F1 val 0.9600 ± 0.0010 so với T00 0.9710 ± 0.0042: vượt nhiễu (&gt;2σ)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Day 2 lab: bonus work (DINOv2 linear probe, distribution shift, Grad-CAM, ONNX), val only
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/submissions/2A202602985_ngo_duc_chung/results.xlsx
+++ b/submissions/2A202602985_ngo_duc_chung/results.xlsx
@@ -15,6 +15,9 @@
     <sheet name="Latency" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Summary" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Lab2_Slide" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Bonus_DINOv2" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Bonus_Shift" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Bonus_ONNX" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1072,6 +1075,398 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>điều kiện ảnh val</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>hiệu chuẩn</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>macro_f1</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>top1</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ece</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>nll</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>sạch</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>chưa hiệu chuẩn (T=1)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>0.9706778541417536</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>0.9768637532133676</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>0.0059104070073552</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0.08284398513763939</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>sạch</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>đã hiệu chuẩn (T=1.049, khớp trên val sạch)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>0.9706778541417536</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>0.9768637532133676</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>0.0063339744495622</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0.0826444991738458</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>tối</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>chưa hiệu chuẩn (T=1)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>0.918582886171966</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>0.930876892316481</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>0.0098524845186676</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>0.1997841233814052</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>tối</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>đã hiệu chuẩn (T=1.049, khớp trên val sạch)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>0.918582886171966</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>0.930876892316481</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>0.0085273619622013</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0.1998896680298524</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>mờ</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>chưa hiệu chuẩn (T=1)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>0.3477643866749061</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>0.6146815195658384</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>0.2770015857877875</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>1.4860387433331</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>mờ</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>đã hiệu chuẩn (T=1.049, khớp trên val sạch)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>0.3477643866749061</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>0.6146815195658384</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>0.2687353815781823</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>1.434048939788929</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>nhiễu</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>chưa hiệu chuẩn (T=1)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>0.8579657759626971</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>0.884318766066838</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>0.0367321949176407</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>0.3617185417195415</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>nhiễu</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>đã hiệu chuẩn (T=1.049, khớp trên val sạch)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>0.8579657759626971</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>0.884318766066838</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>0.032067302382416</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>0.3562180978783958</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="29" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>runtime</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>p50</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>p95</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>p99</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>max|Δ logit| so với PyTorch</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>torch</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>onnxruntime</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PyTorch FP32 (CPU)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>80.4692654999144</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>85.67231649999485</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>98.241255550031</v>
+      </c>
+      <c r="E2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>9.5367431640625e-07</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>1.30.0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>batch 1, ảnh 224, 4 CPU, warmup 10, 100 lần đo, không tính tiền xử lý; file .onnx 111 MB không nộp</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ONNX Runtime FP32 (CPU)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>65.59375799997724</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>68.07489414993597</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>70.2150227500465</v>
+      </c>
+      <c r="E3" t="n">
+        <v>100</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>9.5367431640625e-07</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1.30.0</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>batch 1, ảnh 224, 4 CPU, warmup 10, 100 lần đo, không tính tiền xử lý; file .onnx 111 MB không nộp</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -7084,4 +7479,162 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>exp_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>backbone</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>pretrained_tag</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>init</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>params_m</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>val_macro_f1</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>val_top1</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>val_ece</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>best_epoch</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>sec_per_epoch</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BON_DINO</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>vit_small_patch14_dinov2.lvd142m</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>lvd142m</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>frozen</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>21.632265</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0.8743031732292634</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0.8983147672093688</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>0.0274531433944559</v>
+      </c>
+      <c r="I2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>16.75318224629996</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BON_F01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>in12k_ft_in1k</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>finetune</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>27.827049</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0.9703751013622062</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0.9765781205369894</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0.0056629257382553</v>
+      </c>
+      <c r="I3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>51.96531700069996</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Day 2 lab: bonus multi-fold run (final config on folds 1 and 2, test once per fold)
3-fold (seed 0): top-1 0.9781 +/- 0.0020, macro-F1 0.9724 +/- 0.0024.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/submissions/2A202602985_ngo_duc_chung/results.xlsx
+++ b/submissions/2A202602985_ngo_duc_chung/results.xlsx
@@ -18,6 +18,7 @@
     <sheet name="Bonus_DINOv2" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Bonus_Shift" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Bonus_ONNX" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Bonus_Folds" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1467,6 +1468,210 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>fold</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>n_test</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>top1_test</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>macro_f1_test</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>balanced_acc</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>ece_test</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>recall_Chinee_apple</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>recall_Snake_weed</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>F01_seed0_test.csv</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>3507</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.9760479041916168</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.9698959036084575</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.9733985757322223</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.006779354602224141</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.9557522123893806</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.9411764705882353</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>F01f1_seed0_test.csv</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>3503</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.9800171281758493</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.9747297043599344</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.9726744777032211</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.005668223796745593</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.9244444444444444</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.9655172413793104</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>F01f2_seed0_test.csv</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3501</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.9782919165952585</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.9726163040951642</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.9721843526310864</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.004844661273921785</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.9422222222222222</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.9458128078817734</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>mean ± std (3 fold, ddof=1)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0.9781 ± 0.0020</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0.9724 ± 0.0024</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0.9728 ± 0.0006</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0.0058 ± 0.0010</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0.9408 ± 0.0157</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>0.9508 ± 0.0129</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>